<commit_message>
Muncipales, renommage fichiers et corrections
</commit_message>
<xml_diff>
--- a/data/oxfam/administration_oxfam_2026.xlsx
+++ b/data/oxfam/administration_oxfam_2026.xlsx
@@ -5,32 +5,32 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data For Good\IFP Oxfam Projet VS\oxfam\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data For Good\IFP Oxfam Projet Integration\14_IndexFeminisationPouvoir\data\oxfam\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{51ECA2D5-B9C4-4280-BE33-B6606EDDA41C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A10305B1-EACF-45DD-899F-538EFC9E1B54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="972" yWindow="468" windowWidth="20328" windowHeight="9420" firstSheet="4" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="4" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="agences_hautes_autorités" sheetId="1" r:id="rId1"/>
+    <sheet name="agences_hautes_autorites" sheetId="1" r:id="rId1"/>
     <sheet name="ambassades" sheetId="2" r:id="rId2"/>
     <sheet name="cabinet_premier_ministre" sheetId="3" r:id="rId3"/>
-    <sheet name="cabinet_président" sheetId="4" r:id="rId4"/>
-    <sheet name="dir_cab_ministères" sheetId="5" r:id="rId5"/>
+    <sheet name="cabinet_president" sheetId="4" r:id="rId4"/>
+    <sheet name="dir_cab_ministeres" sheetId="5" r:id="rId5"/>
     <sheet name="gouvernement" sheetId="6" r:id="rId6"/>
-    <sheet name="gouv_postes_régaliens" sheetId="7" r:id="rId7"/>
+    <sheet name="gouv_postes_regaliens" sheetId="7" r:id="rId7"/>
     <sheet name="hautes_juridictions" sheetId="8" r:id="rId8"/>
-    <sheet name="préfectures" sheetId="9" r:id="rId9"/>
+    <sheet name="prefectures" sheetId="9" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">agences_hautes_autorités!$A$1:$H$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">agences_hautes_autorites!$A$1:$H$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">ambassades!$A$1:$H$202</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">cabinet_premier_ministre!$A$1:$H$71</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">cabinet_président!$A$1:$H$57</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">dir_cab_ministères!$A$1:$H$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">cabinet_president!$A$1:$H$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">dir_cab_ministeres!$A$1:$H$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">gouvernement!$A$1:$H$38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">préfectures!$A$1:$I$113</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">prefectures!$A$1:$I$113</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>

</xml_diff>